<commit_message>
Updated Code After Regression
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Czechia_Regression_PK17.xlsx
+++ b/Data/Hires/Workday_NewHire_Czechia_Regression_PK17.xlsx
@@ -1,30 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{B9455642-526F-4A08-9641-0084BA48857A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet sheetId="2" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -259,7 +244,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10699009</t>
+    <t>10699224</t>
   </si>
   <si>
     <t>Passed</t>
@@ -271,10 +256,10 @@
     <t>Czechia</t>
   </si>
   <si>
-    <t>Otho</t>
-  </si>
-  <si>
-    <t>Kerluke</t>
+    <t>Johathan</t>
+  </si>
+  <si>
+    <t>Crist</t>
   </si>
   <si>
     <t>774 272 784</t>
@@ -412,22 +397,22 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10699010</t>
+    <t>10699225</t>
   </si>
   <si>
     <t>895 Store Management (Sepap Pusube (10573442))</t>
   </si>
   <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Trantow</t>
+    <t>Linnea</t>
+  </si>
+  <si>
+    <t>Rowe</t>
   </si>
   <si>
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 23256195</t>
+    <t>Auto 74531265</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -463,54 +448,54 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="12"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="14"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <u/>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
+      <family val="2"/>
       <sz val="14"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="8">
@@ -522,7 +507,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -567,28 +552,16 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <right style="thin"/>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -933,95 +906,94 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CN17"/>
-  <sheetFormatPr defaultRowHeight="15.6" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="8.90625" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9" style="1" customWidth="1"/>
+    <col min="1" max="1" width="12.1796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="109.7265625" style="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="1" customWidth="1"/>
-    <col min="4" max="4" width="46.88671875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="7.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="13.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="16.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="16.109375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="14.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="6.21875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="46.90625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="7.90625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.90625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="16.81640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="16.08984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14.81640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="6.1796875" style="1" customWidth="1"/>
     <col min="11" max="11" width="15" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.44140625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="12.88671875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.453125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="12.90625" style="1" customWidth="1"/>
     <col min="14" max="14" width="16" style="1" customWidth="1"/>
     <col min="15" max="15" width="20" style="1" customWidth="1"/>
-    <col min="16" max="16" width="9.21875" style="1" customWidth="1"/>
-    <col min="17" max="17" width="12.6640625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="6.21875" style="1" customWidth="1"/>
-    <col min="19" max="19" width="8.33203125" style="1" customWidth="1"/>
-    <col min="20" max="20" width="6.21875" style="1" customWidth="1"/>
-    <col min="21" max="21" width="12.109375" style="1" customWidth="1"/>
-    <col min="22" max="22" width="15.6640625" style="1" customWidth="1"/>
-    <col min="23" max="23" width="6.21875" style="1" customWidth="1"/>
-    <col min="24" max="24" width="10.109375" style="1" customWidth="1"/>
-    <col min="25" max="25" width="8.5546875" style="1" customWidth="1"/>
-    <col min="26" max="26" width="22.21875" style="1" customWidth="1"/>
-    <col min="27" max="27" width="16.5546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="9.1796875" style="1" customWidth="1"/>
+    <col min="17" max="17" width="12.6328125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="6.1796875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="8.36328125" style="1" customWidth="1"/>
+    <col min="20" max="20" width="6.1796875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="12.08984375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="15.6328125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="6.1796875" style="1" customWidth="1"/>
+    <col min="24" max="24" width="10.08984375" style="1" customWidth="1"/>
+    <col min="25" max="25" width="8.54296875" style="1" customWidth="1"/>
+    <col min="26" max="26" width="22.1796875" style="1" customWidth="1"/>
+    <col min="27" max="27" width="16.54296875" style="1" customWidth="1"/>
     <col min="28" max="28" width="37" style="1" customWidth="1"/>
-    <col min="29" max="29" width="11.5546875" style="1" customWidth="1"/>
-    <col min="30" max="30" width="21.44140625" style="1" customWidth="1"/>
-    <col min="31" max="31" width="14.6640625" style="1" customWidth="1"/>
-    <col min="32" max="32" width="11.88671875" style="1" customWidth="1"/>
-    <col min="33" max="33" width="26.21875" style="1" customWidth="1"/>
-    <col min="34" max="34" width="23.21875" style="1" customWidth="1"/>
-    <col min="35" max="35" width="23.33203125" style="1" customWidth="1"/>
-    <col min="36" max="36" width="7.21875" style="1" customWidth="1"/>
-    <col min="37" max="37" width="18.77734375" style="1" customWidth="1"/>
-    <col min="38" max="38" width="23.33203125" style="1" customWidth="1"/>
-    <col min="39" max="39" width="23.109375" style="1" customWidth="1"/>
-    <col min="40" max="40" width="18.33203125" style="1" customWidth="1"/>
-    <col min="41" max="41" width="23.5546875" style="1" customWidth="1"/>
-    <col min="42" max="42" width="20.6640625" style="1" customWidth="1"/>
-    <col min="43" max="43" width="20.109375" style="1" customWidth="1"/>
-    <col min="44" max="44" width="10.6640625" style="1" customWidth="1"/>
+    <col min="29" max="29" width="11.54296875" style="1" customWidth="1"/>
+    <col min="30" max="30" width="21.453125" style="1" customWidth="1"/>
+    <col min="31" max="31" width="14.6328125" style="1" customWidth="1"/>
+    <col min="32" max="32" width="11.90625" style="1" customWidth="1"/>
+    <col min="33" max="33" width="26.1796875" style="1" customWidth="1"/>
+    <col min="34" max="34" width="23.1796875" style="1" customWidth="1"/>
+    <col min="35" max="35" width="23.36328125" style="1" customWidth="1"/>
+    <col min="36" max="36" width="7.1796875" style="1" customWidth="1"/>
+    <col min="37" max="37" width="18.81640625" style="1" customWidth="1"/>
+    <col min="38" max="38" width="23.36328125" style="1" customWidth="1"/>
+    <col min="39" max="39" width="23.08984375" style="1" customWidth="1"/>
+    <col min="40" max="40" width="18.36328125" style="1" customWidth="1"/>
+    <col min="41" max="41" width="23.54296875" style="1" customWidth="1"/>
+    <col min="42" max="42" width="20.6328125" style="1" customWidth="1"/>
+    <col min="43" max="43" width="20.08984375" style="1" customWidth="1"/>
+    <col min="44" max="44" width="10.6328125" style="1" customWidth="1"/>
     <col min="45" max="45" width="19" style="1" customWidth="1"/>
-    <col min="46" max="46" width="15.77734375" style="1" customWidth="1"/>
-    <col min="47" max="47" width="13.6640625" style="1" customWidth="1"/>
-    <col min="48" max="48" width="17.77734375" style="1" customWidth="1"/>
-    <col min="49" max="49" width="10.6640625" style="1" customWidth="1"/>
+    <col min="46" max="46" width="15.81640625" style="1" customWidth="1"/>
+    <col min="47" max="47" width="13.6328125" style="1" customWidth="1"/>
+    <col min="48" max="48" width="17.81640625" style="1" customWidth="1"/>
+    <col min="49" max="49" width="10.6328125" style="1" customWidth="1"/>
     <col min="50" max="50" width="19" style="1" customWidth="1"/>
-    <col min="51" max="51" width="14.33203125" style="1" customWidth="1"/>
-    <col min="52" max="52" width="13.6640625" style="1" customWidth="1"/>
-    <col min="53" max="53" width="17.77734375" style="1" customWidth="1"/>
-    <col min="54" max="54" width="8.5546875" style="1" customWidth="1"/>
-    <col min="55" max="55" width="13.6640625" style="1" customWidth="1"/>
-    <col min="56" max="56" width="12.5546875" style="1" customWidth="1"/>
-    <col min="57" max="57" width="14.5546875" style="1" customWidth="1"/>
-    <col min="58" max="58" width="18.88671875" style="1" customWidth="1"/>
-    <col min="59" max="59" width="12.33203125" style="1" customWidth="1"/>
+    <col min="51" max="51" width="14.36328125" style="1" customWidth="1"/>
+    <col min="52" max="52" width="13.6328125" style="1" customWidth="1"/>
+    <col min="53" max="53" width="17.81640625" style="1" customWidth="1"/>
+    <col min="54" max="54" width="8.54296875" style="1" customWidth="1"/>
+    <col min="55" max="55" width="13.6328125" style="1" customWidth="1"/>
+    <col min="56" max="56" width="12.54296875" style="1" customWidth="1"/>
+    <col min="57" max="57" width="14.54296875" style="1" customWidth="1"/>
+    <col min="58" max="58" width="18.90625" style="1" customWidth="1"/>
+    <col min="59" max="59" width="12.36328125" style="1" customWidth="1"/>
     <col min="60" max="60" width="15" style="1" customWidth="1"/>
     <col min="61" max="61" width="26" style="1" customWidth="1"/>
-    <col min="62" max="62" width="25.77734375" style="1" customWidth="1"/>
-    <col min="63" max="63" width="9.44140625" style="1" customWidth="1"/>
-    <col min="64" max="64" width="8.21875" style="1" customWidth="1"/>
-    <col min="65" max="65" width="8.33203125" style="1" customWidth="1"/>
-    <col min="66" max="66" width="17.88671875" style="1" customWidth="1"/>
-    <col min="67" max="67" width="22.88671875" style="1" customWidth="1"/>
-    <col min="68" max="68" width="15.109375" style="1" customWidth="1"/>
-    <col min="69" max="69" width="20.109375" style="1" customWidth="1"/>
-    <col min="70" max="70" width="19.6640625" style="1" customWidth="1"/>
-    <col min="71" max="71" width="29.88671875" style="1" customWidth="1"/>
-    <col min="72" max="72" width="23.44140625" style="1" customWidth="1"/>
-    <col min="73" max="73" width="26.77734375" style="1" customWidth="1"/>
-    <col min="74" max="74" width="30.6640625" style="1" customWidth="1"/>
-    <col min="75" max="75" width="31.5546875" style="1" customWidth="1"/>
-    <col min="76" max="76" width="28.109375" style="1" customWidth="1"/>
+    <col min="62" max="62" width="25.81640625" style="1" customWidth="1"/>
+    <col min="63" max="63" width="9.453125" style="1" customWidth="1"/>
+    <col min="64" max="64" width="8.1796875" style="1" customWidth="1"/>
+    <col min="65" max="65" width="8.36328125" style="1" customWidth="1"/>
+    <col min="66" max="66" width="17.90625" style="1" customWidth="1"/>
+    <col min="67" max="67" width="22.90625" style="1" customWidth="1"/>
+    <col min="68" max="68" width="15.08984375" style="1" customWidth="1"/>
+    <col min="69" max="69" width="20.08984375" style="1" customWidth="1"/>
+    <col min="70" max="70" width="19.6328125" style="1" customWidth="1"/>
+    <col min="71" max="71" width="29.90625" style="1" customWidth="1"/>
+    <col min="72" max="72" width="23.453125" style="1" customWidth="1"/>
+    <col min="73" max="73" width="26.81640625" style="1" customWidth="1"/>
+    <col min="74" max="74" width="30.6328125" style="1" customWidth="1"/>
+    <col min="75" max="75" width="31.54296875" style="1" customWidth="1"/>
+    <col min="76" max="76" width="28.08984375" style="1" customWidth="1"/>
     <col min="77" max="77" width="15" style="1" customWidth="1"/>
-    <col min="78" max="78" width="33.6640625" style="1" customWidth="1"/>
-    <col min="79" max="79" width="26.88671875" style="1" customWidth="1"/>
-    <col min="80" max="80" width="8.88671875" style="1" customWidth="1"/>
-    <col min="81" max="16384" width="8.88671875" style="1"/>
+    <col min="78" max="78" width="33.6328125" style="1" customWidth="1"/>
+    <col min="79" max="79" width="26.90625" style="1" customWidth="1"/>
+    <col min="80" max="16384" width="8.90625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:92" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="18" customHeight="1" spans="1:92" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1273,7 +1245,7 @@
       <c r="CM1" s="1"/>
       <c r="CN1" s="1"/>
     </row>
-    <row r="2" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>75</v>
       </c>
@@ -1383,9 +1355,9 @@
       <c r="AJ2" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="AK2" s="13" t="str">
+      <c r="AK2" s="13">
         <f t="shared" ref="AK2:AK3" si="1">AH2</f>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AL2" s="13">
         <f t="shared" ref="AL2:AL3" si="2">K2</f>
@@ -1415,7 +1387,7 @@
         <v>104</v>
       </c>
       <c r="AT2" s="18">
-        <v>9361110759</v>
+        <v>9461110780</v>
       </c>
       <c r="AU2" s="13" t="s">
         <v>105</v>
@@ -1430,7 +1402,7 @@
         <v>107</v>
       </c>
       <c r="AY2" s="19">
-        <v>141743023</v>
+        <v>142743080</v>
       </c>
       <c r="AZ2" s="13" t="s">
         <v>105</v>
@@ -1517,7 +1489,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="3" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>126</v>
       </c>
@@ -1627,9 +1599,9 @@
       <c r="AJ3" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="AK3" s="13" t="str">
+      <c r="AK3" s="13">
         <f t="shared" si="1"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AL3" s="13">
         <f t="shared" si="2"/>
@@ -1659,7 +1631,7 @@
         <v>104</v>
       </c>
       <c r="AT3" s="18">
-        <v>9361115170</v>
+        <v>9461115182</v>
       </c>
       <c r="AU3" s="13" t="s">
         <v>105</v>
@@ -1674,7 +1646,7 @@
         <v>107</v>
       </c>
       <c r="AY3" s="19">
-        <v>141733024</v>
+        <v>142733082</v>
       </c>
       <c r="AZ3" s="13" t="s">
         <v>105</v>
@@ -1761,7 +1733,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="4" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -1842,7 +1814,7 @@
       <c r="BZ4" s="20"/>
       <c r="CA4" s="20"/>
     </row>
-    <row r="5" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1923,7 +1895,7 @@
       <c r="BZ5" s="20"/>
       <c r="CA5" s="20"/>
     </row>
-    <row r="6" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -2004,7 +1976,7 @@
       <c r="BZ6" s="20"/>
       <c r="CA6" s="20"/>
     </row>
-    <row r="7" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
       <c r="B7" s="21"/>
       <c r="C7" s="8"/>
@@ -2085,7 +2057,7 @@
       <c r="BZ7" s="20"/>
       <c r="CA7" s="20"/>
     </row>
-    <row r="8" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
       <c r="B8" s="9"/>
       <c r="C8" s="8"/>
@@ -2166,7 +2138,7 @@
       <c r="BZ8" s="20"/>
       <c r="CA8" s="20"/>
     </row>
-    <row r="9" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="21"/>
       <c r="C9" s="8"/>
@@ -2247,7 +2219,7 @@
       <c r="BZ9" s="20"/>
       <c r="CA9" s="20"/>
     </row>
-    <row r="10" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -2328,7 +2300,7 @@
       <c r="BZ10" s="20"/>
       <c r="CA10" s="20"/>
     </row>
-    <row r="11" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -2409,7 +2381,7 @@
       <c r="BZ11" s="20"/>
       <c r="CA11" s="20"/>
     </row>
-    <row r="12" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
       <c r="B12" s="21"/>
       <c r="C12" s="8"/>
@@ -2490,7 +2462,7 @@
       <c r="BZ12" s="20"/>
       <c r="CA12" s="20"/>
     </row>
-    <row r="13" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="21"/>
       <c r="C13" s="8"/>
@@ -2571,7 +2543,7 @@
       <c r="BZ13" s="20"/>
       <c r="CA13" s="20"/>
     </row>
-    <row r="14" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8"/>
       <c r="B14" s="21"/>
       <c r="C14" s="8"/>
@@ -2652,7 +2624,7 @@
       <c r="BZ14" s="20"/>
       <c r="CA14" s="20"/>
     </row>
-    <row r="15" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="9"/>
       <c r="C15" s="8"/>
@@ -2733,7 +2705,7 @@
       <c r="BZ15" s="20"/>
       <c r="CA15" s="20"/>
     </row>
-    <row r="16" spans="1:92" s="7" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" ht="15.65" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8"/>
       <c r="B16" s="9"/>
       <c r="C16" s="8"/>
@@ -2814,26 +2786,50 @@
       <c r="BZ16" s="20"/>
       <c r="CA16" s="20"/>
     </row>
-    <row r="17" spans="46:51" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="15.65" customHeight="1" spans="46:51" x14ac:dyDescent="0.25">
       <c r="AT17" s="19"/>
       <c r="AY17" s="19"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ10:AJ16 Y10:Y16 W10:W16 T10:T16" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="12">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ10:AJ16">
       <formula1>INDIRECT($D1)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ16 Y2:Y16 W2:W16 T2:T16" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ16">
       <formula1>INDIRECT($D1)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH10:BH16 J10:J16" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH10:BH16">
       <formula1>INDIRECT($D2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2:BH16 J2:J16" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2:BH16">
       <formula1>INDIRECT($D2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J10:J16">
+      <formula1>INDIRECT($D2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J16">
+      <formula1>INDIRECT($D2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T10:T16">
+      <formula1>INDIRECT($D1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T16">
+      <formula1>INDIRECT($D1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W10:W16">
+      <formula1>INDIRECT($D1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W16">
+      <formula1>INDIRECT($D1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y10:Y16">
+      <formula1>INDIRECT($D1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2:Y16">
+      <formula1>INDIRECT($D1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Czechia job changes script added
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Czechia_Regression_PK17.xlsx
+++ b/Data/Hires/Workday_NewHire_Czechia_Regression_PK17.xlsx
@@ -1,15 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{ACEAF16D-87D6-4ADA-8F06-7E3B0E9E9B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="2" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -244,7 +259,7 @@
     <t>Test1</t>
   </si>
   <si>
-    <t>10699732</t>
+    <t>10700311</t>
   </si>
   <si>
     <t>Passed</t>
@@ -256,10 +271,10 @@
     <t>Czechia</t>
   </si>
   <si>
-    <t>Alessandro</t>
-  </si>
-  <si>
-    <t>Mayert</t>
+    <t>Lizeth</t>
+  </si>
+  <si>
+    <t>Harvey</t>
   </si>
   <si>
     <t>774 272 784</t>
@@ -397,22 +412,22 @@
     <t>Test2</t>
   </si>
   <si>
-    <t>10699735</t>
+    <t>10700312</t>
   </si>
   <si>
     <t>895 Store Management (Sepap Pusube (10573442))</t>
   </si>
   <si>
-    <t>Blake</t>
-  </si>
-  <si>
-    <t>Wunsch</t>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Rippin</t>
   </si>
   <si>
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 7050893</t>
+    <t>Auto 82117314</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -448,57 +463,57 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="12"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="14"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
       <family val="1"/>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
-      <family val="2"/>
       <sz val="14"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -507,7 +522,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.7999816888943144"/>
+        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -530,6 +545,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
@@ -547,16 +567,28 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin"/>
-      <top style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -581,6 +613,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -594,7 +629,7 @@
     <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -608,14 +643,11 @@
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -895,10 +927,10 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:CN4"/>
-  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="8.90625" customHeight="1"/>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:CN11"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="15.65" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.1796875" style="1" customWidth="1"/>
     <col min="2" max="2" width="109.7265625" style="1" customWidth="1"/>
@@ -945,7 +977,7 @@
     <col min="43" max="43" width="20.08984375" style="1" customWidth="1"/>
     <col min="44" max="44" width="10.6328125" style="1" customWidth="1"/>
     <col min="45" max="45" width="19" style="1" customWidth="1"/>
-    <col min="46" max="46" width="15.81640625" style="1" customWidth="1"/>
+    <col min="46" max="46" width="24.81640625" style="1" customWidth="1"/>
     <col min="47" max="47" width="13.6328125" style="1" customWidth="1"/>
     <col min="48" max="48" width="17.81640625" style="1" customWidth="1"/>
     <col min="49" max="49" width="10.6328125" style="1" customWidth="1"/>
@@ -979,10 +1011,11 @@
     <col min="77" max="77" width="15" style="1" customWidth="1"/>
     <col min="78" max="78" width="33.6328125" style="1" customWidth="1"/>
     <col min="79" max="79" width="26.90625" style="1" customWidth="1"/>
-    <col min="80" max="16384" width="8.90625" style="1" customWidth="1"/>
+    <col min="80" max="80" width="8.90625" style="1" customWidth="1"/>
+    <col min="81" max="16384" width="8.90625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" spans="1:92" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:92" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1234,84 +1267,85 @@
       <c r="CM1" s="1"/>
       <c r="CN1" s="1"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="9" t="s">
         <v>76</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="J2" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="K2" s="12">
-        <v>45597</v>
-      </c>
-      <c r="L2" s="10" t="s">
+      <c r="K2" s="13">
+        <f ca="1">TODAY()-40</f>
+        <v>45820</v>
+      </c>
+      <c r="L2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="N2" s="10">
+      <c r="N2" s="11">
         <v>1</v>
       </c>
-      <c r="O2" s="13">
+      <c r="O2" s="14">
         <v>213111231</v>
       </c>
-      <c r="P2" s="11" t="s">
+      <c r="P2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="R2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="S2" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="T2" s="11" t="s">
+      <c r="T2" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="U2" s="12" t="s">
+      <c r="U2" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="V2" s="14" t="s">
+      <c r="V2" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="W2" s="11" t="s">
+      <c r="W2" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="X2" s="12">
-        <f t="shared" ref="X2:X3" si="0">K2</f>
-        <v>45597</v>
-      </c>
-      <c r="Y2" s="11" t="s">
+      <c r="X2" s="13">
+        <f t="shared" ref="X2:X3" ca="1" si="0">K2</f>
+        <v>45820</v>
+      </c>
+      <c r="Y2" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="Z2" s="11" t="s">
+      <c r="Z2" s="12" t="s">
         <v>92</v>
       </c>
       <c r="AA2" s="8" t="s">
@@ -1323,239 +1357,242 @@
       <c r="AC2" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="AD2" s="10" t="s">
+      <c r="AD2" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="AE2" s="10" t="s">
+      <c r="AE2" s="11" t="s">
         <v>97</v>
       </c>
       <c r="AF2" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="AG2" s="15">
+      <c r="AG2" s="16">
         <v>20</v>
       </c>
-      <c r="AH2" s="12" t="s">
+      <c r="AH2" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="AI2" s="11" t="s">
+      <c r="AI2" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="AJ2" s="11" t="s">
+      <c r="AJ2" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="AK2" s="12">
+      <c r="AK2" s="13" t="str">
         <f t="shared" ref="AK2:AK3" si="1">AH2</f>
-        <v>NaN</v>
-      </c>
-      <c r="AL2" s="12">
-        <f t="shared" ref="AL2:AL3" si="2">K2</f>
-        <v>45597</v>
-      </c>
-      <c r="AM2" s="12">
-        <f t="shared" ref="AM2:AM3" si="3">K2</f>
-        <v>45597</v>
-      </c>
-      <c r="AN2" s="11" t="s">
+        <v>N/A</v>
+      </c>
+      <c r="AL2" s="13">
+        <f t="shared" ref="AL2:AL3" ca="1" si="2">K2</f>
+        <v>45820</v>
+      </c>
+      <c r="AM2" s="13">
+        <f t="shared" ref="AM2:AM3" ca="1" si="3">K2</f>
+        <v>45820</v>
+      </c>
+      <c r="AN2" s="12" t="s">
         <v>102</v>
       </c>
       <c r="AO2" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="AP2" s="10">
+      <c r="AP2" s="11">
         <v>100</v>
       </c>
-      <c r="AQ2" s="12">
-        <f t="shared" ref="AQ2:AQ3" si="4">K2+90</f>
-        <v>45687</v>
-      </c>
-      <c r="AR2" s="10" t="s">
+      <c r="AQ2" s="13">
+        <f t="shared" ref="AQ2:AQ3" ca="1" si="4">K2+90</f>
+        <v>45910</v>
+      </c>
+      <c r="AR2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="AS2" s="16" t="s">
+      <c r="AS2" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="AT2" s="17">
-        <v>9461110909</v>
-      </c>
-      <c r="AU2" s="12" t="s">
+      <c r="AT2" s="1">
+        <f t="array" aca="1" ref="AT2:AT3" ca="1">_xlfn.RANDARRAY(2,1,123456789,999999999,TRUE)</f>
+        <v>527090294</v>
+      </c>
+      <c r="AU2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="AV2" s="12" t="s">
+      <c r="AV2" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="AW2" s="10" t="s">
+      <c r="AW2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="AX2" s="16" t="s">
+      <c r="AX2" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="AY2" s="18">
-        <v>152733408</v>
-      </c>
-      <c r="AZ2" s="12" t="s">
+      <c r="AY2" s="1">
+        <f t="array" aca="1" ref="AY2:AY3" ca="1">_xlfn.RANDARRAY(2,1,1234567891,9999999999,TRUE)</f>
+        <v>3199657070</v>
+      </c>
+      <c r="AZ2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="BA2" s="12" t="s">
+      <c r="BA2" s="13" t="s">
         <v>106</v>
       </c>
       <c r="BB2" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="BC2" s="12">
+      <c r="BC2" s="13">
         <v>34284</v>
       </c>
-      <c r="BD2" s="16" t="s">
+      <c r="BD2" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="BE2" s="16" t="s">
+      <c r="BE2" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="BF2" s="16" t="s">
+      <c r="BF2" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="BG2" s="10" t="s">
+      <c r="BG2" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="BH2" s="10" t="s">
+      <c r="BH2" s="11" t="s">
         <v>112</v>
       </c>
       <c r="BI2" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="BJ2" s="16" t="s">
+      <c r="BJ2" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="BK2" s="13" t="s">
+      <c r="BK2" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="BL2" s="13" t="s">
+      <c r="BL2" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="BM2" s="13" t="s">
+      <c r="BM2" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="BN2" s="13" t="s">
+      <c r="BN2" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="BO2" s="13">
+      <c r="BO2" s="14">
         <v>2024</v>
       </c>
-      <c r="BP2" s="13" t="s">
+      <c r="BP2" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="BQ2" s="13">
+      <c r="BQ2" s="14">
         <v>2021</v>
       </c>
-      <c r="BR2" s="13">
+      <c r="BR2" s="14">
         <v>2024</v>
       </c>
-      <c r="BS2" s="13" t="s">
+      <c r="BS2" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="BT2" s="13" t="s">
+      <c r="BT2" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="BU2" s="13" t="s">
+      <c r="BU2" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="BV2" s="19" t="s">
+      <c r="BV2" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="BW2" s="19" t="s">
+      <c r="BW2" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="BX2" s="19">
+      <c r="BX2" s="18">
         <v>213</v>
       </c>
-      <c r="BY2" s="19" t="s">
+      <c r="BY2" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="BZ2" s="19" t="s">
+      <c r="BZ2" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="CA2" s="19" t="s">
+      <c r="CA2" s="18" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="9" t="s">
         <v>127</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="11" t="s">
         <v>79</v>
       </c>
       <c r="F3" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="I3" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="K3" s="12">
-        <v>45597</v>
-      </c>
-      <c r="L3" s="10" t="s">
+      <c r="K3" s="13">
+        <f ca="1">TODAY()-40</f>
+        <v>45820</v>
+      </c>
+      <c r="L3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="M3" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="N3" s="10">
+      <c r="N3" s="11">
         <v>1</v>
       </c>
-      <c r="O3" s="13">
+      <c r="O3" s="14">
         <v>213111231</v>
       </c>
-      <c r="P3" s="11" t="s">
+      <c r="P3" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="Q3" s="11" t="s">
+      <c r="Q3" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="R3" s="11" t="s">
+      <c r="R3" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="S3" s="11" t="s">
+      <c r="S3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="T3" s="11" t="s">
+      <c r="T3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="U3" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="V3" s="14" t="s">
+      <c r="V3" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="W3" s="11" t="s">
+      <c r="W3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="X3" s="12">
-        <f t="shared" si="0"/>
-        <v>45597</v>
-      </c>
-      <c r="Y3" s="11" t="s">
+      <c r="X3" s="13">
+        <f t="shared" ca="1" si="0"/>
+        <v>45820</v>
+      </c>
+      <c r="Y3" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="Z3" s="11" t="s">
+      <c r="Z3" s="12" t="s">
         <v>132</v>
       </c>
       <c r="AA3" s="8" t="s">
@@ -1567,187 +1604,191 @@
       <c r="AC3" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="AD3" s="10" t="s">
+      <c r="AD3" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="AE3" s="10" t="s">
+      <c r="AE3" s="11" t="s">
         <v>97</v>
       </c>
       <c r="AF3" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="AG3" s="15">
+      <c r="AG3" s="16">
         <v>40</v>
       </c>
-      <c r="AH3" s="12" t="s">
+      <c r="AH3" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="AI3" s="11" t="s">
+      <c r="AI3" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="AJ3" s="11" t="s">
+      <c r="AJ3" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="AK3" s="12">
+      <c r="AK3" s="13" t="str">
         <f t="shared" si="1"/>
-        <v>NaN</v>
-      </c>
-      <c r="AL3" s="12">
-        <f t="shared" si="2"/>
-        <v>45597</v>
-      </c>
-      <c r="AM3" s="12">
-        <f t="shared" si="3"/>
-        <v>45597</v>
-      </c>
-      <c r="AN3" s="11" t="s">
+        <v>N/A</v>
+      </c>
+      <c r="AL3" s="13">
+        <f t="shared" ca="1" si="2"/>
+        <v>45820</v>
+      </c>
+      <c r="AM3" s="13">
+        <f t="shared" ca="1" si="3"/>
+        <v>45820</v>
+      </c>
+      <c r="AN3" s="12" t="s">
         <v>136</v>
       </c>
       <c r="AO3" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="AP3" s="10">
+      <c r="AP3" s="11">
         <v>100</v>
       </c>
-      <c r="AQ3" s="12">
-        <f t="shared" si="4"/>
-        <v>45687</v>
-      </c>
-      <c r="AR3" s="10" t="s">
+      <c r="AQ3" s="13">
+        <f t="shared" ca="1" si="4"/>
+        <v>45910</v>
+      </c>
+      <c r="AR3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="AS3" s="16" t="s">
+      <c r="AS3" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="AT3" s="17">
-        <v>9461110910</v>
-      </c>
-      <c r="AU3" s="12" t="s">
+      <c r="AT3" s="1">
+        <f ca="1"/>
+        <v>237778441</v>
+      </c>
+      <c r="AU3" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="AV3" s="12" t="s">
+      <c r="AV3" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="AW3" s="10" t="s">
+      <c r="AW3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="AX3" s="16" t="s">
+      <c r="AX3" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="AY3" s="18">
-        <v>152733409</v>
-      </c>
-      <c r="AZ3" s="12" t="s">
+      <c r="AY3" s="1">
+        <f ca="1"/>
+        <v>4764345306</v>
+      </c>
+      <c r="AZ3" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="BA3" s="12" t="s">
+      <c r="BA3" s="13" t="s">
         <v>106</v>
       </c>
       <c r="BB3" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="BC3" s="12">
+      <c r="BC3" s="13">
         <v>34284</v>
       </c>
-      <c r="BD3" s="16" t="s">
+      <c r="BD3" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="BE3" s="16" t="s">
+      <c r="BE3" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="BF3" s="16" t="s">
+      <c r="BF3" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="BG3" s="10" t="s">
+      <c r="BG3" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="BH3" s="10" t="s">
+      <c r="BH3" s="11" t="s">
         <v>112</v>
       </c>
       <c r="BI3" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="BJ3" s="16" t="s">
+      <c r="BJ3" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="BK3" s="13" t="s">
+      <c r="BK3" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="BL3" s="13" t="s">
+      <c r="BL3" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="BM3" s="13" t="s">
+      <c r="BM3" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="BN3" s="13" t="s">
+      <c r="BN3" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="BO3" s="13">
+      <c r="BO3" s="14">
         <v>2000</v>
       </c>
-      <c r="BP3" s="13" t="s">
+      <c r="BP3" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="BQ3" s="13">
+      <c r="BQ3" s="14">
         <v>1995</v>
       </c>
-      <c r="BR3" s="13">
+      <c r="BR3" s="14">
         <v>2000</v>
       </c>
-      <c r="BS3" s="13" t="s">
+      <c r="BS3" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="BT3" s="13" t="s">
+      <c r="BT3" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="BU3" s="13" t="s">
+      <c r="BU3" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="BV3" s="19" t="s">
+      <c r="BV3" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="BW3" s="19" t="s">
+      <c r="BW3" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="BX3" s="19">
+      <c r="BX3" s="18">
         <v>201</v>
       </c>
-      <c r="BY3" s="19" t="s">
+      <c r="BY3" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="BZ3" s="19" t="s">
+      <c r="BZ3" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="CA3" s="19" t="s">
+      <c r="CA3" s="18" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="4" ht="15.65" customHeight="1" spans="46:51" x14ac:dyDescent="0.25">
-      <c r="AT4" s="18"/>
-      <c r="AY4" s="18"/>
+    <row r="6" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AT6" s="19"/>
+    </row>
+    <row r="7" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AT7" s="19"/>
+    </row>
+    <row r="8" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AT8" s="19"/>
+    </row>
+    <row r="9" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AT9" s="19"/>
+    </row>
+    <row r="10" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AT10" s="19"/>
+    </row>
+    <row r="11" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AT11" s="19"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ3">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ3 Y2:Y3 W2:W3 T2:T3" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($D1)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2:BH3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2:BH3 J2:J3" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT($D2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J3">
-      <formula1>INDIRECT($D2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T3">
-      <formula1>INDIRECT($D1)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W3">
-      <formula1>INDIRECT($D1)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2:Y3">
-      <formula1>INDIRECT($D1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Code added for SMart recruiter.
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Czechia_Regression_PK17.xlsx
+++ b/Data/Hires/Workday_NewHire_Czechia_Regression_PK17.xlsx
@@ -1,35 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{9B464D86-AC80-43A7-A633-ABDD9962DD58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet sheetId="2" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="144">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -259,16 +244,22 @@
     <t>Test1</t>
   </si>
   <si>
+    <t>10700383</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
     <t>895 Retail Team 1 (Sepap Pusube (10573442) (Inherited))</t>
   </si>
   <si>
     <t>Czechia</t>
   </si>
   <si>
-    <t>Hector</t>
-  </si>
-  <si>
-    <t>Sipes</t>
+    <t>Maybell</t>
+  </si>
+  <si>
+    <t>Glover</t>
   </si>
   <si>
     <t>774 272 784</t>
@@ -406,19 +397,32 @@
     <t>Test2</t>
   </si>
   <si>
+    <t xml:space="preserve">Test failed for 'Camille Green' Employee:{10700385}Error: locator.click: Element is not visible
+Call log:
+  [2m- waiting for getByLabel('All Items').first()[22m
+[2m  -   locator resolved to &lt;button class="css-2qog38" aria-current="true" aria-labe…&gt;…&lt;/button&gt;[22m
+[2m  - attempting click action[22m
+[2m  -   scrolling into view if needed[22m
+[2m  -   done scrolling[22m
+</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
     <t>895 Store Management (Sepap Pusube (10573442))</t>
   </si>
   <si>
-    <t>Libbie</t>
-  </si>
-  <si>
-    <t>Zulauf</t>
+    <t>Camille</t>
+  </si>
+  <si>
+    <t>Green</t>
   </si>
   <si>
     <t>775 272 784</t>
   </si>
   <si>
-    <t>Auto 79220054</t>
+    <t>Auto 38684102</t>
   </si>
   <si>
     <t>Team Manager - Retail_NEW</t>
@@ -454,57 +458,57 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Calibri"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="12"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="14"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <u/>
+      <color theme="1"/>
+      <family val="1"/>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
+      <family val="2"/>
       <sz val="14"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -513,7 +517,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -527,11 +531,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -558,28 +557,16 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
+      <right style="thin"/>
+      <top style="thin"/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -604,7 +591,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -620,7 +607,7 @@
     <xf numFmtId="14" fontId="4" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -918,10 +905,10 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:CN11"/>
-  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="15.65" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="8.90625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.1796875" style="1" customWidth="1"/>
     <col min="2" max="2" width="109.7265625" style="1" customWidth="1"/>
@@ -1002,11 +989,10 @@
     <col min="77" max="77" width="15" style="1" customWidth="1"/>
     <col min="78" max="78" width="33.6328125" style="1" customWidth="1"/>
     <col min="79" max="79" width="26.90625" style="1" customWidth="1"/>
-    <col min="80" max="80" width="8.90625" style="1" customWidth="1"/>
-    <col min="81" max="16384" width="8.90625" style="1"/>
+    <col min="80" max="16384" width="8.90625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:92" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="18" customHeight="1" spans="1:92" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1258,42 +1244,46 @@
       <c r="CM1" s="1"/>
       <c r="CN1" s="1"/>
     </row>
-    <row r="2" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" ht="15" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="8"/>
+      <c r="B2" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>77</v>
+      </c>
       <c r="D2" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G2" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="I2" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="J2" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="13">
+        <f>TODAY()-40</f>
+        <v>45826</v>
+      </c>
+      <c r="L2" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="I2" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="J2" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="K2" s="13">
-        <f ca="1">TODAY()-40</f>
-        <v>45823</v>
-      </c>
-      <c r="L2" s="11" t="s">
-        <v>77</v>
-      </c>
       <c r="M2" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="N2" s="11">
         <v>1</v>
@@ -1302,170 +1292,170 @@
         <v>213111231</v>
       </c>
       <c r="P2" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q2" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="R2" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="S2" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="T2" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="Q2" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="R2" s="12" t="s">
+      <c r="U2" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="V2" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="W2" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="S2" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="T2" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="U2" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="V2" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="W2" s="12" t="s">
-        <v>82</v>
-      </c>
       <c r="X2" s="13">
-        <f t="shared" ref="X2:X3" ca="1" si="0">K2</f>
-        <v>45823</v>
+        <f t="shared" ref="X2:X3" si="0">K2</f>
+        <v>45826</v>
       </c>
       <c r="Y2" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Z2" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="AA2" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AB2" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="AC2" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="AD2" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AE2" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AF2" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="AG2" s="16">
         <v>20</v>
       </c>
       <c r="AH2" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AI2" s="12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AJ2" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="AK2" s="13" t="str">
+        <v>101</v>
+      </c>
+      <c r="AK2" s="13">
         <f t="shared" ref="AK2:AK3" si="1">AH2</f>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AL2" s="13">
-        <f t="shared" ref="AL2:AL3" ca="1" si="2">K2</f>
-        <v>45823</v>
+        <f t="shared" ref="AL2:AL3" si="2">K2</f>
+        <v>45826</v>
       </c>
       <c r="AM2" s="13">
-        <f t="shared" ref="AM2:AM3" ca="1" si="3">K2</f>
-        <v>45823</v>
+        <f t="shared" ref="AM2:AM3" si="3">K2</f>
+        <v>45826</v>
       </c>
       <c r="AN2" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="AO2" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AP2" s="11">
         <v>100</v>
       </c>
       <c r="AQ2" s="13">
-        <f t="shared" ref="AQ2:AQ3" ca="1" si="4">K2+90</f>
-        <v>45913</v>
+        <f t="shared" ref="AQ2:AQ3" si="4">K2+90</f>
+        <v>45916</v>
       </c>
       <c r="AR2" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AS2" s="17" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AT2" s="1">
-        <f t="array" aca="1" ref="AT2:AT3" ca="1">_xlfn.RANDARRAY(2,1,123456789,999999999,TRUE)</f>
-        <v>170894114</v>
+        <f t="array" ref="AT2:AT3">_xlfn.RANDARRAY(2,1,123456789,999999999,TRUE)</f>
+        <v>141339042</v>
       </c>
       <c r="AU2" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AV2" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AW2" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AX2" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="AY2" s="1">
+        <f t="array" ref="AY2:AY3">_xlfn.RANDARRAY(2,1,1234567891,9999999999,TRUE)</f>
+        <v>5809444761</v>
+      </c>
+      <c r="AZ2" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="AY2" s="1">
-        <f t="array" aca="1" ref="AY2:AY3" ca="1">_xlfn.RANDARRAY(2,1,1234567891,9999999999,TRUE)</f>
-        <v>8661797469</v>
-      </c>
-      <c r="AZ2" s="13" t="s">
-        <v>103</v>
-      </c>
       <c r="BA2" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BB2" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BC2" s="13">
         <v>34284</v>
       </c>
       <c r="BD2" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="BE2" s="17" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BF2" s="17" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BG2" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BH2" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BI2" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BJ2" s="17" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BK2" s="14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BL2" s="14" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="BM2" s="14" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="BN2" s="14" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="BO2" s="14">
         <v>2024</v>
       </c>
       <c r="BP2" s="14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="BQ2" s="14">
         <v>2021</v>
@@ -1474,69 +1464,73 @@
         <v>2024</v>
       </c>
       <c r="BS2" s="14" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="BT2" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="BU2" s="14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BV2" s="18" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="BW2" s="18" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="BX2" s="18">
         <v>213</v>
       </c>
       <c r="BY2" s="18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="BZ2" s="18" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="CA2" s="18" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
-    <row r="3" spans="1:92" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" ht="15" customHeight="1" spans="1:79" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B3" s="9"/>
-      <c r="C3" s="8"/>
+        <v>126</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>128</v>
+      </c>
       <c r="D3" s="10" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K3" s="13">
-        <f ca="1">TODAY()-40</f>
-        <v>45823</v>
+        <f>TODAY()-40</f>
+        <v>45826</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="M3" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="N3" s="11">
         <v>1</v>
@@ -1545,170 +1539,168 @@
         <v>213111231</v>
       </c>
       <c r="P3" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q3" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="R3" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="S3" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="T3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="Q3" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="R3" s="12" t="s">
+      <c r="U3" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="V3" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="W3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="S3" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="T3" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="U3" s="13" t="s">
-        <v>87</v>
-      </c>
-      <c r="V3" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="W3" s="12" t="s">
-        <v>82</v>
-      </c>
       <c r="X3" s="13">
-        <f t="shared" ca="1" si="0"/>
-        <v>45823</v>
+        <f t="shared" si="0"/>
+        <v>45826</v>
       </c>
       <c r="Y3" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="Z3" s="12" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="AA3" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="AB3" s="8" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="AC3" s="8" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="AD3" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="AE3" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="AF3" s="8" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="AG3" s="16">
         <v>40</v>
       </c>
       <c r="AH3" s="13" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="AI3" s="12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="AJ3" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="AK3" s="13" t="str">
+        <v>101</v>
+      </c>
+      <c r="AK3" s="13">
         <f t="shared" si="1"/>
-        <v>N/A</v>
+        <v>NaN</v>
       </c>
       <c r="AL3" s="13">
-        <f t="shared" ca="1" si="2"/>
-        <v>45823</v>
+        <f t="shared" si="2"/>
+        <v>45826</v>
       </c>
       <c r="AM3" s="13">
-        <f t="shared" ca="1" si="3"/>
-        <v>45823</v>
+        <f t="shared" si="3"/>
+        <v>45826</v>
       </c>
       <c r="AN3" s="12" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="AO3" s="8" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="AP3" s="11">
         <v>100</v>
       </c>
       <c r="AQ3" s="13">
-        <f t="shared" ca="1" si="4"/>
-        <v>45913</v>
+        <f t="shared" si="4"/>
+        <v>45916</v>
       </c>
       <c r="AR3" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AS3" s="17" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="AT3" s="1">
-        <f ca="1"/>
-        <v>489566039</v>
+        <v>621499496</v>
       </c>
       <c r="AU3" s="13" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="AV3" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AW3" s="11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="AX3" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="AY3" s="1">
+        <v>7105135880</v>
+      </c>
+      <c r="AZ3" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="AY3" s="1">
-        <f ca="1"/>
-        <v>6311834980</v>
-      </c>
-      <c r="AZ3" s="13" t="s">
-        <v>103</v>
-      </c>
       <c r="BA3" s="13" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="BB3" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="BC3" s="13">
         <v>34284</v>
       </c>
       <c r="BD3" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="BE3" s="17" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="BF3" s="17" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="BG3" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="BH3" s="11" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="BI3" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="BJ3" s="17" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="BK3" s="14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BL3" s="14" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="BM3" s="14" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="BN3" s="14" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="BO3" s="14">
         <v>2000</v>
       </c>
       <c r="BP3" s="14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="BQ3" s="14">
         <v>1995</v>
@@ -1717,61 +1709,73 @@
         <v>2000</v>
       </c>
       <c r="BS3" s="14" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="BT3" s="14" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="BU3" s="14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="BV3" s="18" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="BW3" s="18" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="BX3" s="18">
         <v>201</v>
       </c>
       <c r="BY3" s="18" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="BZ3" s="18" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="CA3" s="18" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
-    <row r="6" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="15.65" customHeight="1" spans="46:46" x14ac:dyDescent="0.25">
       <c r="AT6" s="19"/>
     </row>
-    <row r="7" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="15.65" customHeight="1" spans="46:46" x14ac:dyDescent="0.25">
       <c r="AT7" s="19"/>
     </row>
-    <row r="8" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="15.65" customHeight="1" spans="46:46" x14ac:dyDescent="0.25">
       <c r="AT8" s="19"/>
     </row>
-    <row r="9" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="15.65" customHeight="1" spans="46:46" x14ac:dyDescent="0.25">
       <c r="AT9" s="19"/>
     </row>
-    <row r="10" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="15.65" customHeight="1" spans="46:46" x14ac:dyDescent="0.25">
       <c r="AT10" s="19"/>
     </row>
-    <row r="11" spans="1:92" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="15.65" customHeight="1" spans="46:46" x14ac:dyDescent="0.25">
       <c r="AT11" s="19"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ3 Y2:Y3 W2:W3 T2:T3" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ2:AJ3">
       <formula1>INDIRECT($D1)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2:BH3 J2:J3" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BH2:BH3">
       <formula1>INDIRECT($D2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J3">
+      <formula1>INDIRECT($D2)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T3">
+      <formula1>INDIRECT($D1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W2:W3">
+      <formula1>INDIRECT($D1)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y2:Y3">
+      <formula1>INDIRECT($D1)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>